<commit_message>
Updated exact 300mm conversion values
</commit_message>
<xml_diff>
--- a/NMR_Rules_Full_Table.xlsx
+++ b/NMR_Rules_Full_Table.xlsx
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>32.8</v>
+        <v>33.333333</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>32.8</v>
+        <v>33.333333</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="G4" t="n">
         <v>2.5</v>
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>32.8</v>
+        <v>33.333333</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -593,10 +593,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="6">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -624,10 +624,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.333333</v>
       </c>
       <c r="G6" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>39.4</v>
+        <v>40</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G7" t="n">
-        <v>6.6</v>
+        <v>6.666667</v>
       </c>
     </row>
     <row r="8">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -686,10 +686,10 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G8" t="n">
-        <v>8.199999999999999</v>
+        <v>8.333333</v>
       </c>
     </row>
     <row r="9">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>39.4</v>
+        <v>40</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G9" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>49.2</v>
+        <v>50</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -748,10 +748,10 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G10" t="n">
-        <v>11.5</v>
+        <v>11.666667</v>
       </c>
     </row>
     <row r="11">
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>49.2</v>
+        <v>50</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -779,10 +779,10 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>13.1</v>
+        <v>13.333333</v>
       </c>
       <c r="G11" t="n">
-        <v>11.5</v>
+        <v>11.666667</v>
       </c>
     </row>
     <row r="12">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -810,10 +810,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G12" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>39.4</v>
+        <v>40</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -841,10 +841,10 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G13" t="n">
-        <v>11.5</v>
+        <v>11.666667</v>
       </c>
     </row>
     <row r="14">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>49.2</v>
+        <v>50</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -872,10 +872,10 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G14" t="n">
-        <v>13.1</v>
+        <v>13.333333</v>
       </c>
     </row>
     <row r="15">
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>49.2</v>
+        <v>50</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -903,10 +903,10 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>13.1</v>
+        <v>13.333333</v>
       </c>
       <c r="G15" t="n">
-        <v>13.1</v>
+        <v>13.333333</v>
       </c>
     </row>
     <row r="16">
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -934,10 +934,10 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G16" t="n">
-        <v>11.5</v>
+        <v>11.666667</v>
       </c>
     </row>
     <row r="17">
@@ -952,7 +952,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>39.4</v>
+        <v>40</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -965,10 +965,10 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G17" t="n">
-        <v>13.1</v>
+        <v>13.333333</v>
       </c>
     </row>
     <row r="18">
@@ -983,7 +983,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>49.2</v>
+        <v>50</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -996,10 +996,10 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G18" t="n">
-        <v>16.4</v>
+        <v>16.666667</v>
       </c>
     </row>
     <row r="19">
@@ -1014,7 +1014,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>49.2</v>
+        <v>50</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1027,10 +1027,10 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>13.1</v>
+        <v>13.333333</v>
       </c>
       <c r="G19" t="n">
-        <v>16.4</v>
+        <v>16.666667</v>
       </c>
     </row>
     <row r="20">
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>59.1</v>
+        <v>60</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1058,10 +1058,10 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G20" t="n">
-        <v>19.7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>59.1</v>
+        <v>60</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1089,10 +1089,10 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>13.1</v>
+        <v>13.333333</v>
       </c>
       <c r="G21" t="n">
-        <v>19.7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>59.1</v>
+        <v>60</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1120,10 +1120,10 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>16.4</v>
+        <v>16.666667</v>
       </c>
       <c r="G22" t="n">
-        <v>19.7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23">
@@ -1138,7 +1138,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>59.1</v>
+        <v>60</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1151,10 +1151,10 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>18</v>
+        <v>18.333333</v>
       </c>
       <c r="G23" t="n">
-        <v>19.7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24">
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1182,10 +1182,10 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G24" t="n">
-        <v>16.4</v>
+        <v>16.666667</v>
       </c>
     </row>
     <row r="25">
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>39.4</v>
+        <v>40</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1213,10 +1213,10 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G25" t="n">
-        <v>18</v>
+        <v>18.333333</v>
       </c>
     </row>
     <row r="26">
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>49.2</v>
+        <v>50</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1244,10 +1244,10 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G26" t="n">
-        <v>19.7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>49.2</v>
+        <v>50</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1275,10 +1275,10 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>13.1</v>
+        <v>13.333333</v>
       </c>
       <c r="G27" t="n">
-        <v>19.7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28">
@@ -1293,7 +1293,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>59.1</v>
+        <v>60</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1306,10 +1306,10 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="G28" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="29">
@@ -1324,7 +1324,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>59.1</v>
+        <v>60</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1337,10 +1337,10 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>13.1</v>
+        <v>13.333333</v>
       </c>
       <c r="G29" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="30">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>59.1</v>
+        <v>60</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1368,10 +1368,10 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>16.4</v>
+        <v>16.666667</v>
       </c>
       <c r="G30" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="31">
@@ -1386,7 +1386,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>59.1</v>
+        <v>60</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1399,10 +1399,10 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>18</v>
+        <v>18.333333</v>
       </c>
       <c r="G31" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="32">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>68.90000000000001</v>
+        <v>70</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1430,10 +1430,10 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
       <c r="G32" t="n">
-        <v>23</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="33">
@@ -1448,7 +1448,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>78.7</v>
+        <v>80</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1461,10 +1461,10 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>26.2</v>
+        <v>26.6</v>
       </c>
       <c r="G33" t="n">
-        <v>26.2</v>
+        <v>26.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>